<commit_message>
Include feedback and complete course history in exported reports
</commit_message>
<xml_diff>
--- a/tests/e2e/fixtures/students.xlsx
+++ b/tests/e2e/fixtures/students.xlsx
@@ -1,6 +1,14 @@
+
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheets>
+    <sheet name="Students" sheetId="1" r:id="rId1"/>
+  </sheets>
+</workbook>
+</file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>שם פרטי</t>
   </si>
@@ -23,7 +31,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>
     <row r="1">
       <c r="A1" t="s">

</xml_diff>